<commit_message>
Update Kerala gold rates
</commit_message>
<xml_diff>
--- a/gold_rates.xlsx
+++ b/gold_rates.xlsx
@@ -49234,6 +49234,14 @@
         <v>14190.0</v>
       </c>
     </row>
+    <row r="6154">
+      <c r="A6154" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="B6154">
+        <v>14190.0</v>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>